<commit_message>
Add audited-value and independent-audit-status disclosures to all 14 executive rollup reports
</commit_message>
<xml_diff>
--- a/00_Executive_Rollup_Report/AMEX_RiskIQ_Platform_Executive_Rollup_Workbook.xlsx
+++ b/00_Executive_Rollup_Report/AMEX_RiskIQ_Platform_Executive_Rollup_Workbook.xlsx
@@ -135,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,6 +169,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -860,6 +861,30 @@
       <c r="B17" s="5" t="inlineStr">
         <is>
           <t>73 / 14 / 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="100" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Business Impact — Modeled Estimate, Not Audited Value</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Problem 14's executive rollup computes a modeled net-value estimate of $429.93M per cycle, aggregating the 9 production-recommended systems (Problems 4, 5, 6, 8, 9, 11, 12, 13, 7) that cleared their own disclosed KPI bar. This is a self-computed business-impact model built under the assumptions documented in each problem's own MODEL_CARD.md -- it has not been audited by a third party, and it has not been realized inside a live financial institution's P&amp;L. Problems 1-2 (foundational), Problem 3 ($4.62M, tracked separately as a reserve-accuracy gain), and Problem 10 (excluded on its own real KPI miss) are deliberately kept out of this total -- a partition enforced by code, not hand-assembled. See the 'Financial Methodology' sheet for full per-problem assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Independent Audit Status</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>This project was developed as an independent portfolio body of work and has not undergone formal validation, audit, or sign-off by a financial institution's model risk management (SR 11-7 or equivalent) function, a third-party auditor, or a regulator. All model outputs, risk metrics, and business-impact figures in this report are self-computed under the assumptions stated herein and have not been realized in a live production environment at a financial institution.</t>
         </is>
       </c>
     </row>

</xml_diff>